<commit_message>
Update leaves.xlsx from Google Sheet
</commit_message>
<xml_diff>
--- a/data/leaves.xlsx
+++ b/data/leaves.xlsx
@@ -5,13 +5,15 @@
   <sheets>
     <sheet state="visible" name="الاجازات" sheetId="1" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'الاجازات'!$A$1:$N$997</definedName>
+  </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8424" uniqueCount="1403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8546" uniqueCount="1515">
   <si>
     <t>leave_id</t>
   </si>
@@ -682,7 +684,7 @@
     <t>LV-79</t>
   </si>
   <si>
-    <t>راشد الشريهي</t>
+    <t>راشد فائز سويحل الشمري</t>
   </si>
   <si>
     <t>RASHID ALSHERIHI</t>
@@ -4168,18 +4170,165 @@
     <t>LV-837</t>
   </si>
   <si>
+    <t>LV-838</t>
+  </si>
+  <si>
+    <t>LV-839</t>
+  </si>
+  <si>
+    <t>LV-840</t>
+  </si>
+  <si>
     <t>فيصل سعد عبدالله الشمري</t>
   </si>
   <si>
     <t>FAISAL SAAD ALSHAMMARI</t>
   </si>
   <si>
+    <t>LV-841</t>
+  </si>
+  <si>
+    <t>LV-842</t>
+  </si>
+  <si>
+    <t>LV-843</t>
+  </si>
+  <si>
+    <t>LV-844</t>
+  </si>
+  <si>
+    <t>LV-845</t>
+  </si>
+  <si>
+    <t>LV-846</t>
+  </si>
+  <si>
+    <t>LV-847</t>
+  </si>
+  <si>
+    <t>LV-848</t>
+  </si>
+  <si>
+    <t>LV-849</t>
+  </si>
+  <si>
+    <t>LV-850</t>
+  </si>
+  <si>
+    <t>LV-851</t>
+  </si>
+  <si>
+    <t>LV-852</t>
+  </si>
+  <si>
+    <t>LV-853</t>
+  </si>
+  <si>
+    <t>LV-854</t>
+  </si>
+  <si>
+    <t>LV-855</t>
+  </si>
+  <si>
+    <t>LV-856</t>
+  </si>
+  <si>
+    <t>LV-857</t>
+  </si>
+  <si>
+    <t>LV-858</t>
+  </si>
+  <si>
+    <t>LV-859</t>
+  </si>
+  <si>
+    <t>LV-860</t>
+  </si>
+  <si>
     <t>Industrial Engineer - مهندس صناعي</t>
   </si>
   <si>
+    <t>LV-861</t>
+  </si>
+  <si>
+    <t>LV-862</t>
+  </si>
+  <si>
+    <t>LV-863</t>
+  </si>
+  <si>
+    <t>LV-864</t>
+  </si>
+  <si>
+    <t>LV-865</t>
+  </si>
+  <si>
+    <t>LV-866</t>
+  </si>
+  <si>
+    <t>LV-867</t>
+  </si>
+  <si>
+    <t>LV-868</t>
+  </si>
+  <si>
+    <t>LV-869</t>
+  </si>
+  <si>
+    <t>LV-870</t>
+  </si>
+  <si>
+    <t>LV-871</t>
+  </si>
+  <si>
+    <t>LV-872</t>
+  </si>
+  <si>
+    <t>LV-873</t>
+  </si>
+  <si>
+    <t>LV-874</t>
+  </si>
+  <si>
+    <t>LV-875</t>
+  </si>
+  <si>
+    <t>LV-876</t>
+  </si>
+  <si>
+    <t>LV-877</t>
+  </si>
+  <si>
+    <t>LV-878</t>
+  </si>
+  <si>
+    <t>LV-879</t>
+  </si>
+  <si>
     <t>NAWAF NAWAR ALOTAIBI</t>
   </si>
   <si>
+    <t>LV-880</t>
+  </si>
+  <si>
+    <t>LV-881</t>
+  </si>
+  <si>
+    <t>LV-882</t>
+  </si>
+  <si>
+    <t>LV-883</t>
+  </si>
+  <si>
+    <t>LV-884</t>
+  </si>
+  <si>
+    <t>LV-885</t>
+  </si>
+  <si>
+    <t>LV-886</t>
+  </si>
+  <si>
     <t>هتان سليمان الغازي</t>
   </si>
   <si>
@@ -4189,7 +4338,130 @@
     <t>GN | Procurement</t>
   </si>
   <si>
-    <t>راشد فائز سويحل الشمري</t>
+    <t>LV-887</t>
+  </si>
+  <si>
+    <t>LV-888</t>
+  </si>
+  <si>
+    <t>LV-889</t>
+  </si>
+  <si>
+    <t>LV-890</t>
+  </si>
+  <si>
+    <t>LV-891</t>
+  </si>
+  <si>
+    <t>LV-892</t>
+  </si>
+  <si>
+    <t>LV-893</t>
+  </si>
+  <si>
+    <t>LV-894</t>
+  </si>
+  <si>
+    <t>LV-895</t>
+  </si>
+  <si>
+    <t>LV-896</t>
+  </si>
+  <si>
+    <t>LV-897</t>
+  </si>
+  <si>
+    <t>LV-898</t>
+  </si>
+  <si>
+    <t>LV-899</t>
+  </si>
+  <si>
+    <t>LV-900</t>
+  </si>
+  <si>
+    <t>LV-901</t>
+  </si>
+  <si>
+    <t>LV-902</t>
+  </si>
+  <si>
+    <t>LV-903</t>
+  </si>
+  <si>
+    <t>LV-904</t>
+  </si>
+  <si>
+    <t>LV-905</t>
+  </si>
+  <si>
+    <t>LV-906</t>
+  </si>
+  <si>
+    <t>LV-907</t>
+  </si>
+  <si>
+    <t>LV-908</t>
+  </si>
+  <si>
+    <t>LV-909</t>
+  </si>
+  <si>
+    <t>LV-910</t>
+  </si>
+  <si>
+    <t>LV-911</t>
+  </si>
+  <si>
+    <t>LV-912</t>
+  </si>
+  <si>
+    <t>LV-913</t>
+  </si>
+  <si>
+    <t>LV-914</t>
+  </si>
+  <si>
+    <t>LV-915</t>
+  </si>
+  <si>
+    <t>LV-916</t>
+  </si>
+  <si>
+    <t>LV-917</t>
+  </si>
+  <si>
+    <t>LV-918</t>
+  </si>
+  <si>
+    <t>LV-919</t>
+  </si>
+  <si>
+    <t>LV-920</t>
+  </si>
+  <si>
+    <t>LV-921</t>
+  </si>
+  <si>
+    <t>LV-922</t>
+  </si>
+  <si>
+    <t>LV-923</t>
+  </si>
+  <si>
+    <t>LV-924</t>
+  </si>
+  <si>
+    <t>LV-925</t>
+  </si>
+  <si>
+    <t>LV-926</t>
+  </si>
+  <si>
+    <t>LV-927</t>
+  </si>
+  <si>
+    <t>LV-928</t>
   </si>
   <si>
     <t>محمد ريان خالد</t>
@@ -4198,28 +4470,94 @@
     <t>MD RAIYAN KHALID</t>
   </si>
   <si>
+    <t>LV-929</t>
+  </si>
+  <si>
     <t>هوم بهادور كومال</t>
   </si>
   <si>
     <t>HUM BAHADUR KUMAL</t>
   </si>
   <si>
+    <t>LV-930</t>
+  </si>
+  <si>
+    <t>LV-931</t>
+  </si>
+  <si>
     <t>دابلو كومار</t>
   </si>
   <si>
     <t>DABLU KUMAR</t>
   </si>
   <si>
+    <t>LV-932</t>
+  </si>
+  <si>
     <t>نانو بينوا</t>
   </si>
   <si>
     <t>NANU THANKAPPAN BINU</t>
   </si>
   <si>
+    <t>LV-933</t>
+  </si>
+  <si>
     <t>جوهر الاسلام كالو مياه</t>
   </si>
   <si>
     <t>JOHIRUL ISLAM KALU MIAH</t>
+  </si>
+  <si>
+    <t>LV-934</t>
+  </si>
+  <si>
+    <t>LV-935</t>
+  </si>
+  <si>
+    <t>LV-936</t>
+  </si>
+  <si>
+    <t>LV-937</t>
+  </si>
+  <si>
+    <t>LV-938</t>
+  </si>
+  <si>
+    <t>LV-939</t>
+  </si>
+  <si>
+    <t>LV-940</t>
+  </si>
+  <si>
+    <t>LV-941</t>
+  </si>
+  <si>
+    <t>LV-942</t>
+  </si>
+  <si>
+    <t>LV-943</t>
+  </si>
+  <si>
+    <t>LV-944</t>
+  </si>
+  <si>
+    <t>LV-945</t>
+  </si>
+  <si>
+    <t>LV-946</t>
+  </si>
+  <si>
+    <t>LV-947</t>
+  </si>
+  <si>
+    <t>LV-948</t>
+  </si>
+  <si>
+    <t>LV-949</t>
+  </si>
+  <si>
+    <t>LV-950</t>
   </si>
 </sst>
 </file>
@@ -4534,6 +4872,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:N997" displayName="جدول_1" name="جدول_1" id="1">
+  <autoFilter ref="$A$1:$N$997"/>
   <tableColumns count="14">
     <tableColumn name="leave_id" id="1"/>
     <tableColumn name="employee_id" id="2"/>
@@ -40137,14 +40476,24 @@
       <c r="A805" s="6" t="s">
         <v>1350</v>
       </c>
-      <c r="B805" s="17"/>
-      <c r="C805" s="14"/>
+      <c r="B805" s="8">
+        <v>30497.0</v>
+      </c>
+      <c r="C805" s="14">
+        <v>30497.0</v>
+      </c>
       <c r="D805" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="E805" s="15"/>
-      <c r="F805" s="15"/>
-      <c r="G805" s="15"/>
+      <c r="E805" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="F805" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="G805" s="16" t="s">
+        <v>1209</v>
+      </c>
       <c r="H805" s="10" t="s">
         <v>19</v>
       </c>
@@ -40171,14 +40520,24 @@
       <c r="A806" s="6" t="s">
         <v>1351</v>
       </c>
-      <c r="B806" s="17"/>
-      <c r="C806" s="14"/>
+      <c r="B806" s="8">
+        <v>30497.0</v>
+      </c>
+      <c r="C806" s="14">
+        <v>30497.0</v>
+      </c>
       <c r="D806" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="E806" s="15"/>
-      <c r="F806" s="15"/>
-      <c r="G806" s="15"/>
+      <c r="E806" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="F806" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="G806" s="16" t="s">
+        <v>1209</v>
+      </c>
       <c r="H806" s="10" t="s">
         <v>19</v>
       </c>
@@ -40205,14 +40564,24 @@
       <c r="A807" s="6" t="s">
         <v>1352</v>
       </c>
-      <c r="B807" s="17"/>
-      <c r="C807" s="14"/>
+      <c r="B807" s="8">
+        <v>30497.0</v>
+      </c>
+      <c r="C807" s="14">
+        <v>30497.0</v>
+      </c>
       <c r="D807" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="E807" s="15"/>
-      <c r="F807" s="15"/>
-      <c r="G807" s="15"/>
+      <c r="E807" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="F807" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="G807" s="16" t="s">
+        <v>1209</v>
+      </c>
       <c r="H807" s="10" t="s">
         <v>19</v>
       </c>
@@ -41292,7 +41661,9 @@
       <c r="R831" s="7"/>
     </row>
     <row r="832" ht="18.0" customHeight="1">
-      <c r="A832" s="6"/>
+      <c r="A832" s="6" t="s">
+        <v>1385</v>
+      </c>
       <c r="B832" s="8">
         <v>27943.0</v>
       </c>
@@ -41334,7 +41705,9 @@
       <c r="R832" s="7"/>
     </row>
     <row r="833" ht="18.0" customHeight="1">
-      <c r="A833" s="6"/>
+      <c r="A833" s="6" t="s">
+        <v>1386</v>
+      </c>
       <c r="B833" s="8">
         <v>27943.0</v>
       </c>
@@ -41376,7 +41749,9 @@
       <c r="R833" s="7"/>
     </row>
     <row r="834" ht="18.0" customHeight="1">
-      <c r="A834" s="6"/>
+      <c r="A834" s="6" t="s">
+        <v>1387</v>
+      </c>
       <c r="B834" s="8">
         <v>27509.0</v>
       </c>
@@ -41384,10 +41759,10 @@
         <v>27509.0</v>
       </c>
       <c r="D834" s="9" t="s">
-        <v>1385</v>
+        <v>1388</v>
       </c>
       <c r="E834" s="16" t="s">
-        <v>1386</v>
+        <v>1389</v>
       </c>
       <c r="F834" s="16" t="s">
         <v>597</v>
@@ -41418,7 +41793,9 @@
       <c r="R834" s="7"/>
     </row>
     <row r="835" ht="18.0" customHeight="1">
-      <c r="A835" s="6"/>
+      <c r="A835" s="6" t="s">
+        <v>1390</v>
+      </c>
       <c r="B835" s="8">
         <v>27509.0</v>
       </c>
@@ -41426,10 +41803,10 @@
         <v>27509.0</v>
       </c>
       <c r="D835" s="9" t="s">
-        <v>1385</v>
+        <v>1388</v>
       </c>
       <c r="E835" s="16" t="s">
-        <v>1386</v>
+        <v>1389</v>
       </c>
       <c r="F835" s="16" t="s">
         <v>597</v>
@@ -41460,7 +41837,9 @@
       <c r="R835" s="7"/>
     </row>
     <row r="836" ht="18.0" customHeight="1">
-      <c r="A836" s="6"/>
+      <c r="A836" s="6" t="s">
+        <v>1391</v>
+      </c>
       <c r="B836" s="8">
         <v>32083.0</v>
       </c>
@@ -41502,7 +41881,9 @@
       <c r="R836" s="7"/>
     </row>
     <row r="837" ht="18.0" customHeight="1">
-      <c r="A837" s="6"/>
+      <c r="A837" s="6" t="s">
+        <v>1392</v>
+      </c>
       <c r="B837" s="8">
         <v>30576.0</v>
       </c>
@@ -41544,7 +41925,9 @@
       <c r="R837" s="7"/>
     </row>
     <row r="838" ht="18.0" customHeight="1">
-      <c r="A838" s="6"/>
+      <c r="A838" s="6" t="s">
+        <v>1393</v>
+      </c>
       <c r="B838" s="8">
         <v>30560.0</v>
       </c>
@@ -41586,7 +41969,9 @@
       <c r="R838" s="7"/>
     </row>
     <row r="839" ht="18.0" customHeight="1">
-      <c r="A839" s="6"/>
+      <c r="A839" s="6" t="s">
+        <v>1394</v>
+      </c>
       <c r="B839" s="8">
         <v>30560.0</v>
       </c>
@@ -41628,7 +42013,9 @@
       <c r="R839" s="7"/>
     </row>
     <row r="840" ht="18.0" customHeight="1">
-      <c r="A840" s="6"/>
+      <c r="A840" s="6" t="s">
+        <v>1395</v>
+      </c>
       <c r="B840" s="8">
         <v>30560.0</v>
       </c>
@@ -41670,7 +42057,9 @@
       <c r="R840" s="7"/>
     </row>
     <row r="841" ht="18.0" customHeight="1">
-      <c r="A841" s="6"/>
+      <c r="A841" s="6" t="s">
+        <v>1396</v>
+      </c>
       <c r="B841" s="8">
         <v>30536.0</v>
       </c>
@@ -41712,7 +42101,9 @@
       <c r="R841" s="7"/>
     </row>
     <row r="842" ht="18.0" customHeight="1">
-      <c r="A842" s="6"/>
+      <c r="A842" s="6" t="s">
+        <v>1397</v>
+      </c>
       <c r="B842" s="8">
         <v>30536.0</v>
       </c>
@@ -41754,7 +42145,9 @@
       <c r="R842" s="7"/>
     </row>
     <row r="843" ht="18.0" customHeight="1">
-      <c r="A843" s="6"/>
+      <c r="A843" s="6" t="s">
+        <v>1398</v>
+      </c>
       <c r="B843" s="8">
         <v>29446.0</v>
       </c>
@@ -41796,7 +42189,9 @@
       <c r="R843" s="7"/>
     </row>
     <row r="844" ht="18.0" customHeight="1">
-      <c r="A844" s="6"/>
+      <c r="A844" s="6" t="s">
+        <v>1399</v>
+      </c>
       <c r="B844" s="8">
         <v>29446.0</v>
       </c>
@@ -41838,7 +42233,9 @@
       <c r="R844" s="7"/>
     </row>
     <row r="845" ht="18.0" customHeight="1">
-      <c r="A845" s="6"/>
+      <c r="A845" s="6" t="s">
+        <v>1400</v>
+      </c>
       <c r="B845" s="8">
         <v>29446.0</v>
       </c>
@@ -41880,7 +42277,9 @@
       <c r="R845" s="7"/>
     </row>
     <row r="846" ht="18.0" customHeight="1">
-      <c r="A846" s="6"/>
+      <c r="A846" s="6" t="s">
+        <v>1401</v>
+      </c>
       <c r="B846" s="8">
         <v>29446.0</v>
       </c>
@@ -41922,7 +42321,9 @@
       <c r="R846" s="7"/>
     </row>
     <row r="847" ht="18.0" customHeight="1">
-      <c r="A847" s="6"/>
+      <c r="A847" s="6" t="s">
+        <v>1402</v>
+      </c>
       <c r="B847" s="8">
         <v>29446.0</v>
       </c>
@@ -41964,7 +42365,9 @@
       <c r="R847" s="7"/>
     </row>
     <row r="848" ht="18.0" customHeight="1">
-      <c r="A848" s="6"/>
+      <c r="A848" s="6" t="s">
+        <v>1403</v>
+      </c>
       <c r="B848" s="8">
         <v>29446.0</v>
       </c>
@@ -42006,7 +42409,9 @@
       <c r="R848" s="7"/>
     </row>
     <row r="849" ht="18.0" customHeight="1">
-      <c r="A849" s="6"/>
+      <c r="A849" s="6" t="s">
+        <v>1404</v>
+      </c>
       <c r="B849" s="8">
         <v>29442.0</v>
       </c>
@@ -42048,7 +42453,9 @@
       <c r="R849" s="7"/>
     </row>
     <row r="850" ht="18.0" customHeight="1">
-      <c r="A850" s="6"/>
+      <c r="A850" s="6" t="s">
+        <v>1405</v>
+      </c>
       <c r="B850" s="8">
         <v>31731.0</v>
       </c>
@@ -42090,7 +42497,9 @@
       <c r="R850" s="7"/>
     </row>
     <row r="851" ht="18.0" customHeight="1">
-      <c r="A851" s="6"/>
+      <c r="A851" s="6" t="s">
+        <v>1406</v>
+      </c>
       <c r="B851" s="8">
         <v>31731.0</v>
       </c>
@@ -42132,7 +42541,9 @@
       <c r="R851" s="7"/>
     </row>
     <row r="852" ht="18.0" customHeight="1">
-      <c r="A852" s="6"/>
+      <c r="A852" s="6" t="s">
+        <v>1407</v>
+      </c>
       <c r="B852" s="8">
         <v>31731.0</v>
       </c>
@@ -42174,7 +42585,9 @@
       <c r="R852" s="7"/>
     </row>
     <row r="853" ht="18.0" customHeight="1">
-      <c r="A853" s="6"/>
+      <c r="A853" s="6" t="s">
+        <v>1408</v>
+      </c>
       <c r="B853" s="8">
         <v>31731.0</v>
       </c>
@@ -42216,7 +42629,9 @@
       <c r="R853" s="7"/>
     </row>
     <row r="854" ht="18.0" customHeight="1">
-      <c r="A854" s="6"/>
+      <c r="A854" s="6" t="s">
+        <v>1409</v>
+      </c>
       <c r="B854" s="8">
         <v>32877.0</v>
       </c>
@@ -42233,7 +42648,7 @@
         <v>58</v>
       </c>
       <c r="G854" s="18" t="s">
-        <v>1387</v>
+        <v>1410</v>
       </c>
       <c r="H854" s="10" t="s">
         <v>19</v>
@@ -42258,7 +42673,9 @@
       <c r="R854" s="7"/>
     </row>
     <row r="855" ht="18.0" customHeight="1">
-      <c r="A855" s="6"/>
+      <c r="A855" s="6" t="s">
+        <v>1411</v>
+      </c>
       <c r="B855" s="8">
         <v>31354.0</v>
       </c>
@@ -42300,7 +42717,9 @@
       <c r="R855" s="7"/>
     </row>
     <row r="856" ht="18.0" customHeight="1">
-      <c r="A856" s="6"/>
+      <c r="A856" s="6" t="s">
+        <v>1412</v>
+      </c>
       <c r="B856" s="8">
         <v>29977.0</v>
       </c>
@@ -42342,7 +42761,9 @@
       <c r="R856" s="7"/>
     </row>
     <row r="857" ht="18.0" customHeight="1">
-      <c r="A857" s="6"/>
+      <c r="A857" s="6" t="s">
+        <v>1413</v>
+      </c>
       <c r="B857" s="8">
         <v>32877.0</v>
       </c>
@@ -42359,7 +42780,7 @@
         <v>58</v>
       </c>
       <c r="G857" s="18" t="s">
-        <v>1387</v>
+        <v>1410</v>
       </c>
       <c r="H857" s="10" t="s">
         <v>19</v>
@@ -42384,7 +42805,9 @@
       <c r="R857" s="7"/>
     </row>
     <row r="858" ht="18.0" customHeight="1">
-      <c r="A858" s="6"/>
+      <c r="A858" s="6" t="s">
+        <v>1414</v>
+      </c>
       <c r="B858" s="8">
         <v>30584.0</v>
       </c>
@@ -42426,7 +42849,9 @@
       <c r="R858" s="7"/>
     </row>
     <row r="859" ht="18.0" customHeight="1">
-      <c r="A859" s="6"/>
+      <c r="A859" s="6" t="s">
+        <v>1415</v>
+      </c>
       <c r="B859" s="8">
         <v>30584.0</v>
       </c>
@@ -42468,7 +42893,9 @@
       <c r="R859" s="7"/>
     </row>
     <row r="860" ht="18.0" customHeight="1">
-      <c r="A860" s="6"/>
+      <c r="A860" s="6" t="s">
+        <v>1416</v>
+      </c>
       <c r="B860" s="8">
         <v>30584.0</v>
       </c>
@@ -42510,7 +42937,9 @@
       <c r="R860" s="7"/>
     </row>
     <row r="861" ht="18.0" customHeight="1">
-      <c r="A861" s="6"/>
+      <c r="A861" s="6" t="s">
+        <v>1417</v>
+      </c>
       <c r="B861" s="8">
         <v>29862.0</v>
       </c>
@@ -42552,7 +42981,9 @@
       <c r="R861" s="7"/>
     </row>
     <row r="862" ht="18.0" customHeight="1">
-      <c r="A862" s="6"/>
+      <c r="A862" s="6" t="s">
+        <v>1418</v>
+      </c>
       <c r="B862" s="8">
         <v>29862.0</v>
       </c>
@@ -42594,7 +43025,9 @@
       <c r="R862" s="7"/>
     </row>
     <row r="863" ht="18.0" customHeight="1">
-      <c r="A863" s="6"/>
+      <c r="A863" s="6" t="s">
+        <v>1419</v>
+      </c>
       <c r="B863" s="8">
         <v>29858.0</v>
       </c>
@@ -42636,7 +43069,9 @@
       <c r="R863" s="7"/>
     </row>
     <row r="864" ht="18.0" customHeight="1">
-      <c r="A864" s="6"/>
+      <c r="A864" s="6" t="s">
+        <v>1420</v>
+      </c>
       <c r="B864" s="8">
         <v>29858.0</v>
       </c>
@@ -42678,7 +43113,9 @@
       <c r="R864" s="7"/>
     </row>
     <row r="865" ht="18.0" customHeight="1">
-      <c r="A865" s="6"/>
+      <c r="A865" s="6" t="s">
+        <v>1421</v>
+      </c>
       <c r="B865" s="8">
         <v>29858.0</v>
       </c>
@@ -42720,7 +43157,9 @@
       <c r="R865" s="7"/>
     </row>
     <row r="866" ht="18.0" customHeight="1">
-      <c r="A866" s="6"/>
+      <c r="A866" s="6" t="s">
+        <v>1422</v>
+      </c>
       <c r="B866" s="8">
         <v>26390.0</v>
       </c>
@@ -42762,7 +43201,9 @@
       <c r="R866" s="7"/>
     </row>
     <row r="867" ht="18.0" customHeight="1">
-      <c r="A867" s="6"/>
+      <c r="A867" s="6" t="s">
+        <v>1423</v>
+      </c>
       <c r="B867" s="8">
         <v>26390.0</v>
       </c>
@@ -42804,7 +43245,9 @@
       <c r="R867" s="7"/>
     </row>
     <row r="868" ht="18.0" customHeight="1">
-      <c r="A868" s="6"/>
+      <c r="A868" s="6" t="s">
+        <v>1424</v>
+      </c>
       <c r="B868" s="8">
         <v>29628.0</v>
       </c>
@@ -42846,7 +43289,9 @@
       <c r="R868" s="7"/>
     </row>
     <row r="869" ht="18.0" customHeight="1">
-      <c r="A869" s="6"/>
+      <c r="A869" s="6" t="s">
+        <v>1425</v>
+      </c>
       <c r="B869" s="8">
         <v>29448.0</v>
       </c>
@@ -42888,7 +43333,9 @@
       <c r="R869" s="7"/>
     </row>
     <row r="870" ht="18.0" customHeight="1">
-      <c r="A870" s="6"/>
+      <c r="A870" s="6" t="s">
+        <v>1426</v>
+      </c>
       <c r="B870" s="8">
         <v>23613.0</v>
       </c>
@@ -42930,7 +43377,9 @@
       <c r="R870" s="7"/>
     </row>
     <row r="871" ht="18.0" customHeight="1">
-      <c r="A871" s="6"/>
+      <c r="A871" s="6" t="s">
+        <v>1427</v>
+      </c>
       <c r="B871" s="8">
         <v>30361.0</v>
       </c>
@@ -42972,7 +43421,9 @@
       <c r="R871" s="7"/>
     </row>
     <row r="872" ht="18.0" customHeight="1">
-      <c r="A872" s="6"/>
+      <c r="A872" s="6" t="s">
+        <v>1428</v>
+      </c>
       <c r="B872" s="8">
         <v>30361.0</v>
       </c>
@@ -43014,7 +43465,9 @@
       <c r="R872" s="7"/>
     </row>
     <row r="873" ht="18.0" customHeight="1">
-      <c r="A873" s="6"/>
+      <c r="A873" s="6" t="s">
+        <v>1429</v>
+      </c>
       <c r="B873" s="8">
         <v>27941.0</v>
       </c>
@@ -43025,7 +43478,7 @@
         <v>732</v>
       </c>
       <c r="E873" s="16" t="s">
-        <v>1388</v>
+        <v>1430</v>
       </c>
       <c r="F873" s="16" t="s">
         <v>429</v>
@@ -43056,7 +43509,9 @@
       <c r="R873" s="7"/>
     </row>
     <row r="874" ht="18.0" customHeight="1">
-      <c r="A874" s="6"/>
+      <c r="A874" s="6" t="s">
+        <v>1431</v>
+      </c>
       <c r="B874" s="8">
         <v>30361.0</v>
       </c>
@@ -43098,7 +43553,9 @@
       <c r="R874" s="7"/>
     </row>
     <row r="875" ht="18.0" customHeight="1">
-      <c r="A875" s="6"/>
+      <c r="A875" s="6" t="s">
+        <v>1432</v>
+      </c>
       <c r="B875" s="8">
         <v>31283.0</v>
       </c>
@@ -43140,7 +43597,9 @@
       <c r="R875" s="7"/>
     </row>
     <row r="876" ht="18.0" customHeight="1">
-      <c r="A876" s="6"/>
+      <c r="A876" s="6" t="s">
+        <v>1433</v>
+      </c>
       <c r="B876" s="8">
         <v>31283.0</v>
       </c>
@@ -43182,7 +43641,9 @@
       <c r="R876" s="7"/>
     </row>
     <row r="877" ht="18.0" customHeight="1">
-      <c r="A877" s="6"/>
+      <c r="A877" s="6" t="s">
+        <v>1434</v>
+      </c>
       <c r="B877" s="8">
         <v>31283.0</v>
       </c>
@@ -43224,7 +43685,9 @@
       <c r="R877" s="7"/>
     </row>
     <row r="878" ht="18.0" customHeight="1">
-      <c r="A878" s="6"/>
+      <c r="A878" s="6" t="s">
+        <v>1435</v>
+      </c>
       <c r="B878" s="8">
         <v>31283.0</v>
       </c>
@@ -43266,7 +43729,9 @@
       <c r="R878" s="7"/>
     </row>
     <row r="879" ht="18.0" customHeight="1">
-      <c r="A879" s="6"/>
+      <c r="A879" s="6" t="s">
+        <v>1436</v>
+      </c>
       <c r="B879" s="8">
         <v>31283.0</v>
       </c>
@@ -43308,7 +43773,9 @@
       <c r="R879" s="7"/>
     </row>
     <row r="880" ht="18.0" customHeight="1">
-      <c r="A880" s="6"/>
+      <c r="A880" s="6" t="s">
+        <v>1437</v>
+      </c>
       <c r="B880" s="8">
         <v>28875.0</v>
       </c>
@@ -43316,13 +43783,13 @@
         <v>28875.0</v>
       </c>
       <c r="D880" s="9" t="s">
-        <v>1389</v>
+        <v>1438</v>
       </c>
       <c r="E880" s="16" t="s">
-        <v>1390</v>
+        <v>1439</v>
       </c>
       <c r="F880" s="16" t="s">
-        <v>1391</v>
+        <v>1440</v>
       </c>
       <c r="G880" s="16" t="s">
         <v>1209</v>
@@ -43350,7 +43817,9 @@
       <c r="R880" s="7"/>
     </row>
     <row r="881" ht="18.0" customHeight="1">
-      <c r="A881" s="6"/>
+      <c r="A881" s="6" t="s">
+        <v>1441</v>
+      </c>
       <c r="B881" s="8">
         <v>28875.0</v>
       </c>
@@ -43358,13 +43827,13 @@
         <v>28875.0</v>
       </c>
       <c r="D881" s="9" t="s">
-        <v>1389</v>
+        <v>1438</v>
       </c>
       <c r="E881" s="16" t="s">
-        <v>1390</v>
+        <v>1439</v>
       </c>
       <c r="F881" s="16" t="s">
-        <v>1391</v>
+        <v>1440</v>
       </c>
       <c r="G881" s="16" t="s">
         <v>1209</v>
@@ -43392,7 +43861,9 @@
       <c r="R881" s="7"/>
     </row>
     <row r="882" ht="18.0" customHeight="1">
-      <c r="A882" s="6"/>
+      <c r="A882" s="6" t="s">
+        <v>1442</v>
+      </c>
       <c r="B882" s="8">
         <v>27164.0</v>
       </c>
@@ -43434,7 +43905,9 @@
       <c r="R882" s="7"/>
     </row>
     <row r="883" ht="18.0" customHeight="1">
-      <c r="A883" s="6"/>
+      <c r="A883" s="6" t="s">
+        <v>1443</v>
+      </c>
       <c r="B883" s="8">
         <v>32391.0</v>
       </c>
@@ -43476,7 +43949,9 @@
       <c r="R883" s="7"/>
     </row>
     <row r="884" ht="18.0" customHeight="1">
-      <c r="A884" s="6"/>
+      <c r="A884" s="6" t="s">
+        <v>1444</v>
+      </c>
       <c r="B884" s="8">
         <v>31304.0</v>
       </c>
@@ -43518,7 +43993,9 @@
       <c r="R884" s="7"/>
     </row>
     <row r="885" ht="18.0" customHeight="1">
-      <c r="A885" s="6"/>
+      <c r="A885" s="6" t="s">
+        <v>1445</v>
+      </c>
       <c r="B885" s="8">
         <v>30646.0</v>
       </c>
@@ -43560,7 +44037,9 @@
       <c r="R885" s="7"/>
     </row>
     <row r="886" ht="18.0" customHeight="1">
-      <c r="A886" s="6"/>
+      <c r="A886" s="6" t="s">
+        <v>1446</v>
+      </c>
       <c r="B886" s="8">
         <v>31720.0</v>
       </c>
@@ -43602,7 +44081,9 @@
       <c r="R886" s="7"/>
     </row>
     <row r="887" ht="18.0" customHeight="1">
-      <c r="A887" s="6"/>
+      <c r="A887" s="6" t="s">
+        <v>1447</v>
+      </c>
       <c r="B887" s="8">
         <v>31720.0</v>
       </c>
@@ -43644,7 +44125,9 @@
       <c r="R887" s="7"/>
     </row>
     <row r="888" ht="18.0" customHeight="1">
-      <c r="A888" s="6"/>
+      <c r="A888" s="6" t="s">
+        <v>1448</v>
+      </c>
       <c r="B888" s="8">
         <v>31720.0</v>
       </c>
@@ -43686,7 +44169,9 @@
       <c r="R888" s="7"/>
     </row>
     <row r="889" ht="18.0" customHeight="1">
-      <c r="A889" s="6"/>
+      <c r="A889" s="6" t="s">
+        <v>1449</v>
+      </c>
       <c r="B889" s="8">
         <v>31720.0</v>
       </c>
@@ -43728,7 +44213,9 @@
       <c r="R889" s="7"/>
     </row>
     <row r="890" ht="18.0" customHeight="1">
-      <c r="A890" s="6"/>
+      <c r="A890" s="6" t="s">
+        <v>1450</v>
+      </c>
       <c r="B890" s="8">
         <v>31720.0</v>
       </c>
@@ -43770,7 +44257,9 @@
       <c r="R890" s="7"/>
     </row>
     <row r="891" ht="18.0" customHeight="1">
-      <c r="A891" s="6"/>
+      <c r="A891" s="6" t="s">
+        <v>1451</v>
+      </c>
       <c r="B891" s="8">
         <v>30858.0</v>
       </c>
@@ -43812,7 +44301,9 @@
       <c r="R891" s="7"/>
     </row>
     <row r="892" ht="18.0" customHeight="1">
-      <c r="A892" s="6"/>
+      <c r="A892" s="6" t="s">
+        <v>1452</v>
+      </c>
       <c r="B892" s="8">
         <v>30858.0</v>
       </c>
@@ -43854,7 +44345,9 @@
       <c r="R892" s="7"/>
     </row>
     <row r="893" ht="18.0" customHeight="1">
-      <c r="A893" s="6"/>
+      <c r="A893" s="6" t="s">
+        <v>1453</v>
+      </c>
       <c r="B893" s="8">
         <v>30858.0</v>
       </c>
@@ -43896,7 +44389,9 @@
       <c r="R893" s="7"/>
     </row>
     <row r="894" ht="18.0" customHeight="1">
-      <c r="A894" s="6"/>
+      <c r="A894" s="6" t="s">
+        <v>1454</v>
+      </c>
       <c r="B894" s="8">
         <v>30574.0</v>
       </c>
@@ -43938,7 +44433,9 @@
       <c r="R894" s="7"/>
     </row>
     <row r="895" ht="18.0" customHeight="1">
-      <c r="A895" s="6"/>
+      <c r="A895" s="6" t="s">
+        <v>1455</v>
+      </c>
       <c r="B895" s="8">
         <v>30574.0</v>
       </c>
@@ -43980,7 +44477,9 @@
       <c r="R895" s="7"/>
     </row>
     <row r="896" ht="18.0" customHeight="1">
-      <c r="A896" s="6"/>
+      <c r="A896" s="6" t="s">
+        <v>1456</v>
+      </c>
       <c r="B896" s="8">
         <v>30574.0</v>
       </c>
@@ -44022,7 +44521,9 @@
       <c r="R896" s="7"/>
     </row>
     <row r="897" ht="18.0" customHeight="1">
-      <c r="A897" s="6"/>
+      <c r="A897" s="6" t="s">
+        <v>1457</v>
+      </c>
       <c r="B897" s="8">
         <v>28211.0</v>
       </c>
@@ -44064,7 +44565,9 @@
       <c r="R897" s="7"/>
     </row>
     <row r="898" ht="18.0" customHeight="1">
-      <c r="A898" s="6"/>
+      <c r="A898" s="6" t="s">
+        <v>1458</v>
+      </c>
       <c r="B898" s="8">
         <v>28211.0</v>
       </c>
@@ -44106,7 +44609,9 @@
       <c r="R898" s="7"/>
     </row>
     <row r="899" ht="18.0" customHeight="1">
-      <c r="A899" s="6"/>
+      <c r="A899" s="6" t="s">
+        <v>1459</v>
+      </c>
       <c r="B899" s="8">
         <v>28211.0</v>
       </c>
@@ -44148,7 +44653,9 @@
       <c r="R899" s="7"/>
     </row>
     <row r="900" ht="18.0" customHeight="1">
-      <c r="A900" s="6"/>
+      <c r="A900" s="6" t="s">
+        <v>1460</v>
+      </c>
       <c r="B900" s="8">
         <v>28211.0</v>
       </c>
@@ -44190,7 +44697,9 @@
       <c r="R900" s="7"/>
     </row>
     <row r="901" ht="18.0" customHeight="1">
-      <c r="A901" s="6"/>
+      <c r="A901" s="6" t="s">
+        <v>1461</v>
+      </c>
       <c r="B901" s="8">
         <v>29756.0</v>
       </c>
@@ -44232,7 +44741,9 @@
       <c r="R901" s="7"/>
     </row>
     <row r="902" ht="18.0" customHeight="1">
-      <c r="A902" s="6"/>
+      <c r="A902" s="6" t="s">
+        <v>1462</v>
+      </c>
       <c r="B902" s="8">
         <v>27864.0</v>
       </c>
@@ -44274,7 +44785,9 @@
       <c r="R902" s="7"/>
     </row>
     <row r="903" ht="18.0" customHeight="1">
-      <c r="A903" s="6"/>
+      <c r="A903" s="6" t="s">
+        <v>1463</v>
+      </c>
       <c r="B903" s="8">
         <v>28215.0</v>
       </c>
@@ -44316,7 +44829,9 @@
       <c r="R903" s="7"/>
     </row>
     <row r="904" ht="18.0" customHeight="1">
-      <c r="A904" s="6"/>
+      <c r="A904" s="6" t="s">
+        <v>1464</v>
+      </c>
       <c r="B904" s="8">
         <v>31279.0</v>
       </c>
@@ -44358,7 +44873,9 @@
       <c r="R904" s="7"/>
     </row>
     <row r="905" ht="18.0" customHeight="1">
-      <c r="A905" s="6"/>
+      <c r="A905" s="6" t="s">
+        <v>1465</v>
+      </c>
       <c r="B905" s="8">
         <v>31279.0</v>
       </c>
@@ -44400,7 +44917,9 @@
       <c r="R905" s="7"/>
     </row>
     <row r="906" ht="18.0" customHeight="1">
-      <c r="A906" s="6"/>
+      <c r="A906" s="6" t="s">
+        <v>1466</v>
+      </c>
       <c r="B906" s="8">
         <v>31279.0</v>
       </c>
@@ -44442,7 +44961,9 @@
       <c r="R906" s="7"/>
     </row>
     <row r="907" ht="18.0" customHeight="1">
-      <c r="A907" s="6"/>
+      <c r="A907" s="6" t="s">
+        <v>1467</v>
+      </c>
       <c r="B907" s="8">
         <v>31279.0</v>
       </c>
@@ -44484,7 +45005,9 @@
       <c r="R907" s="7"/>
     </row>
     <row r="908" ht="18.0" customHeight="1">
-      <c r="A908" s="6"/>
+      <c r="A908" s="6" t="s">
+        <v>1468</v>
+      </c>
       <c r="B908" s="8">
         <v>31279.0</v>
       </c>
@@ -44526,7 +45049,9 @@
       <c r="R908" s="7"/>
     </row>
     <row r="909" ht="18.0" customHeight="1">
-      <c r="A909" s="6"/>
+      <c r="A909" s="6" t="s">
+        <v>1469</v>
+      </c>
       <c r="B909" s="8">
         <v>31271.0</v>
       </c>
@@ -44564,7 +45089,9 @@
       <c r="R909" s="7"/>
     </row>
     <row r="910" ht="18.0" customHeight="1">
-      <c r="A910" s="6"/>
+      <c r="A910" s="6" t="s">
+        <v>1470</v>
+      </c>
       <c r="B910" s="8">
         <v>31271.0</v>
       </c>
@@ -44602,7 +45129,9 @@
       <c r="R910" s="7"/>
     </row>
     <row r="911" ht="18.0" customHeight="1">
-      <c r="A911" s="6"/>
+      <c r="A911" s="6" t="s">
+        <v>1471</v>
+      </c>
       <c r="B911" s="8">
         <v>30353.0</v>
       </c>
@@ -44644,7 +45173,9 @@
       <c r="R911" s="7"/>
     </row>
     <row r="912" ht="18.0" customHeight="1">
-      <c r="A912" s="6"/>
+      <c r="A912" s="6" t="s">
+        <v>1472</v>
+      </c>
       <c r="B912" s="8">
         <v>32348.0</v>
       </c>
@@ -44686,7 +45217,9 @@
       <c r="R912" s="7"/>
     </row>
     <row r="913" ht="18.0" customHeight="1">
-      <c r="A913" s="6"/>
+      <c r="A913" s="6" t="s">
+        <v>1473</v>
+      </c>
       <c r="B913" s="8">
         <v>32348.0</v>
       </c>
@@ -44728,7 +45261,9 @@
       <c r="R913" s="7"/>
     </row>
     <row r="914" ht="18.0" customHeight="1">
-      <c r="A914" s="6"/>
+      <c r="A914" s="6" t="s">
+        <v>1474</v>
+      </c>
       <c r="B914" s="8">
         <v>31962.0</v>
       </c>
@@ -44770,7 +45305,9 @@
       <c r="R914" s="7"/>
     </row>
     <row r="915" ht="18.0" customHeight="1">
-      <c r="A915" s="6"/>
+      <c r="A915" s="6" t="s">
+        <v>1475</v>
+      </c>
       <c r="B915" s="8">
         <v>31962.0</v>
       </c>
@@ -44812,7 +45349,9 @@
       <c r="R915" s="7"/>
     </row>
     <row r="916" ht="18.0" customHeight="1">
-      <c r="A916" s="6"/>
+      <c r="A916" s="6" t="s">
+        <v>1476</v>
+      </c>
       <c r="B916" s="8">
         <v>31962.0</v>
       </c>
@@ -44854,7 +45393,9 @@
       <c r="R916" s="7"/>
     </row>
     <row r="917" ht="18.0" customHeight="1">
-      <c r="A917" s="6"/>
+      <c r="A917" s="6" t="s">
+        <v>1477</v>
+      </c>
       <c r="B917" s="8">
         <v>30497.0</v>
       </c>
@@ -44862,7 +45403,7 @@
         <v>30497.0</v>
       </c>
       <c r="D917" s="9" t="s">
-        <v>1392</v>
+        <v>223</v>
       </c>
       <c r="E917" s="16" t="s">
         <v>224</v>
@@ -44896,7 +45437,9 @@
       <c r="R917" s="7"/>
     </row>
     <row r="918" ht="18.0" customHeight="1">
-      <c r="A918" s="6"/>
+      <c r="A918" s="6" t="s">
+        <v>1478</v>
+      </c>
       <c r="B918" s="8">
         <v>30497.0</v>
       </c>
@@ -44904,7 +45447,7 @@
         <v>30497.0</v>
       </c>
       <c r="D918" s="9" t="s">
-        <v>1392</v>
+        <v>223</v>
       </c>
       <c r="E918" s="16" t="s">
         <v>224</v>
@@ -44938,7 +45481,9 @@
       <c r="R918" s="7"/>
     </row>
     <row r="919" ht="18.0" customHeight="1">
-      <c r="A919" s="6"/>
+      <c r="A919" s="6" t="s">
+        <v>1479</v>
+      </c>
       <c r="B919" s="8">
         <v>30497.0</v>
       </c>
@@ -44946,7 +45491,7 @@
         <v>30497.0</v>
       </c>
       <c r="D919" s="9" t="s">
-        <v>1392</v>
+        <v>223</v>
       </c>
       <c r="E919" s="16" t="s">
         <v>224</v>
@@ -44980,7 +45525,9 @@
       <c r="R919" s="7"/>
     </row>
     <row r="920" ht="18.0" customHeight="1">
-      <c r="A920" s="6"/>
+      <c r="A920" s="6" t="s">
+        <v>1480</v>
+      </c>
       <c r="B920" s="8">
         <v>30497.0</v>
       </c>
@@ -44988,7 +45535,7 @@
         <v>30497.0</v>
       </c>
       <c r="D920" s="9" t="s">
-        <v>1392</v>
+        <v>223</v>
       </c>
       <c r="E920" s="16" t="s">
         <v>224</v>
@@ -45022,7 +45569,9 @@
       <c r="R920" s="7"/>
     </row>
     <row r="921" ht="18.0" customHeight="1">
-      <c r="A921" s="6"/>
+      <c r="A921" s="6" t="s">
+        <v>1481</v>
+      </c>
       <c r="B921" s="8">
         <v>26796.0</v>
       </c>
@@ -45064,7 +45613,9 @@
       <c r="R921" s="7"/>
     </row>
     <row r="922" ht="18.0" customHeight="1">
-      <c r="A922" s="6"/>
+      <c r="A922" s="6" t="s">
+        <v>1482</v>
+      </c>
       <c r="B922" s="8">
         <v>31456.0</v>
       </c>
@@ -45072,10 +45623,10 @@
         <v>31456.0</v>
       </c>
       <c r="D922" s="9" t="s">
-        <v>1393</v>
+        <v>1483</v>
       </c>
       <c r="E922" s="16" t="s">
-        <v>1394</v>
+        <v>1484</v>
       </c>
       <c r="F922" s="16" t="s">
         <v>429</v>
@@ -45106,7 +45657,9 @@
       <c r="R922" s="7"/>
     </row>
     <row r="923" ht="18.0" customHeight="1">
-      <c r="A923" s="6"/>
+      <c r="A923" s="6" t="s">
+        <v>1485</v>
+      </c>
       <c r="B923" s="8">
         <v>27912.0</v>
       </c>
@@ -45114,10 +45667,10 @@
         <v>27912.0</v>
       </c>
       <c r="D923" s="9" t="s">
-        <v>1395</v>
+        <v>1486</v>
       </c>
       <c r="E923" s="16" t="s">
-        <v>1396</v>
+        <v>1487</v>
       </c>
       <c r="F923" s="16" t="s">
         <v>209</v>
@@ -45148,7 +45701,9 @@
       <c r="R923" s="7"/>
     </row>
     <row r="924" ht="18.0" customHeight="1">
-      <c r="A924" s="6"/>
+      <c r="A924" s="6" t="s">
+        <v>1488</v>
+      </c>
       <c r="B924" s="8">
         <v>27912.0</v>
       </c>
@@ -45156,10 +45711,10 @@
         <v>27912.0</v>
       </c>
       <c r="D924" s="9" t="s">
-        <v>1395</v>
+        <v>1486</v>
       </c>
       <c r="E924" s="16" t="s">
-        <v>1396</v>
+        <v>1487</v>
       </c>
       <c r="F924" s="16" t="s">
         <v>209</v>
@@ -45190,7 +45745,9 @@
       <c r="R924" s="7"/>
     </row>
     <row r="925" ht="18.0" customHeight="1">
-      <c r="A925" s="6"/>
+      <c r="A925" s="6" t="s">
+        <v>1489</v>
+      </c>
       <c r="B925" s="8">
         <v>32031.0</v>
       </c>
@@ -45198,10 +45755,10 @@
         <v>32031.0</v>
       </c>
       <c r="D925" s="9" t="s">
-        <v>1397</v>
+        <v>1490</v>
       </c>
       <c r="E925" s="16" t="s">
-        <v>1398</v>
+        <v>1491</v>
       </c>
       <c r="F925" s="16" t="s">
         <v>326</v>
@@ -45232,7 +45789,9 @@
       <c r="R925" s="7"/>
     </row>
     <row r="926" ht="18.0" customHeight="1">
-      <c r="A926" s="6"/>
+      <c r="A926" s="6" t="s">
+        <v>1492</v>
+      </c>
       <c r="B926" s="8">
         <v>17666.0</v>
       </c>
@@ -45240,10 +45799,10 @@
         <v>17666.0</v>
       </c>
       <c r="D926" s="9" t="s">
-        <v>1399</v>
+        <v>1493</v>
       </c>
       <c r="E926" s="16" t="s">
-        <v>1400</v>
+        <v>1494</v>
       </c>
       <c r="F926" s="16" t="s">
         <v>326</v>
@@ -45274,7 +45833,9 @@
       <c r="R926" s="7"/>
     </row>
     <row r="927" ht="18.0" customHeight="1">
-      <c r="A927" s="6"/>
+      <c r="A927" s="6" t="s">
+        <v>1495</v>
+      </c>
       <c r="B927" s="8">
         <v>26226.0</v>
       </c>
@@ -45282,10 +45843,10 @@
         <v>26226.0</v>
       </c>
       <c r="D927" s="9" t="s">
-        <v>1401</v>
+        <v>1496</v>
       </c>
       <c r="E927" s="16" t="s">
-        <v>1402</v>
+        <v>1497</v>
       </c>
       <c r="F927" s="16" t="s">
         <v>326</v>
@@ -45316,7 +45877,9 @@
       <c r="R927" s="7"/>
     </row>
     <row r="928" ht="18.0" customHeight="1">
-      <c r="A928" s="6"/>
+      <c r="A928" s="6" t="s">
+        <v>1498</v>
+      </c>
       <c r="B928" s="8">
         <v>31442.0</v>
       </c>
@@ -45354,7 +45917,9 @@
       <c r="R928" s="7"/>
     </row>
     <row r="929" ht="18.0" customHeight="1">
-      <c r="A929" s="6"/>
+      <c r="A929" s="6" t="s">
+        <v>1499</v>
+      </c>
       <c r="B929" s="8">
         <v>31442.0</v>
       </c>
@@ -45392,7 +45957,9 @@
       <c r="R929" s="7"/>
     </row>
     <row r="930" ht="18.0" customHeight="1">
-      <c r="A930" s="6"/>
+      <c r="A930" s="6" t="s">
+        <v>1500</v>
+      </c>
       <c r="B930" s="8">
         <v>31442.0</v>
       </c>
@@ -45430,7 +45997,9 @@
       <c r="R930" s="7"/>
     </row>
     <row r="931" ht="18.0" customHeight="1">
-      <c r="A931" s="6"/>
+      <c r="A931" s="6" t="s">
+        <v>1501</v>
+      </c>
       <c r="B931" s="8">
         <v>31442.0</v>
       </c>
@@ -45468,7 +46037,9 @@
       <c r="R931" s="7"/>
     </row>
     <row r="932" ht="18.0" customHeight="1">
-      <c r="A932" s="6"/>
+      <c r="A932" s="6" t="s">
+        <v>1502</v>
+      </c>
       <c r="B932" s="17"/>
       <c r="C932" s="14"/>
       <c r="D932" s="22"/>
@@ -45494,7 +46065,9 @@
       <c r="R932" s="7"/>
     </row>
     <row r="933" ht="18.0" customHeight="1">
-      <c r="A933" s="6"/>
+      <c r="A933" s="6" t="s">
+        <v>1503</v>
+      </c>
       <c r="B933" s="17"/>
       <c r="C933" s="14"/>
       <c r="D933" s="22"/>
@@ -45520,7 +46093,9 @@
       <c r="R933" s="7"/>
     </row>
     <row r="934" ht="18.0" customHeight="1">
-      <c r="A934" s="6"/>
+      <c r="A934" s="6" t="s">
+        <v>1504</v>
+      </c>
       <c r="B934" s="17"/>
       <c r="C934" s="14"/>
       <c r="D934" s="22"/>
@@ -45546,7 +46121,9 @@
       <c r="R934" s="7"/>
     </row>
     <row r="935" ht="18.0" customHeight="1">
-      <c r="A935" s="6"/>
+      <c r="A935" s="6" t="s">
+        <v>1505</v>
+      </c>
       <c r="B935" s="17"/>
       <c r="C935" s="14"/>
       <c r="D935" s="22"/>
@@ -45572,7 +46149,9 @@
       <c r="R935" s="7"/>
     </row>
     <row r="936" ht="18.0" customHeight="1">
-      <c r="A936" s="6"/>
+      <c r="A936" s="6" t="s">
+        <v>1506</v>
+      </c>
       <c r="B936" s="17"/>
       <c r="C936" s="14"/>
       <c r="D936" s="22"/>
@@ -45598,7 +46177,9 @@
       <c r="R936" s="7"/>
     </row>
     <row r="937" ht="18.0" customHeight="1">
-      <c r="A937" s="6"/>
+      <c r="A937" s="6" t="s">
+        <v>1507</v>
+      </c>
       <c r="B937" s="17"/>
       <c r="C937" s="14"/>
       <c r="D937" s="22"/>
@@ -45624,7 +46205,9 @@
       <c r="R937" s="7"/>
     </row>
     <row r="938" ht="18.0" customHeight="1">
-      <c r="A938" s="6"/>
+      <c r="A938" s="6" t="s">
+        <v>1508</v>
+      </c>
       <c r="B938" s="17"/>
       <c r="C938" s="14"/>
       <c r="D938" s="22"/>
@@ -45650,7 +46233,9 @@
       <c r="R938" s="7"/>
     </row>
     <row r="939" ht="18.0" customHeight="1">
-      <c r="A939" s="6"/>
+      <c r="A939" s="6" t="s">
+        <v>1509</v>
+      </c>
       <c r="B939" s="17"/>
       <c r="C939" s="14"/>
       <c r="D939" s="22"/>
@@ -45676,7 +46261,9 @@
       <c r="R939" s="7"/>
     </row>
     <row r="940" ht="18.0" customHeight="1">
-      <c r="A940" s="6"/>
+      <c r="A940" s="6" t="s">
+        <v>1510</v>
+      </c>
       <c r="B940" s="17"/>
       <c r="C940" s="14"/>
       <c r="D940" s="22"/>
@@ -45702,7 +46289,9 @@
       <c r="R940" s="7"/>
     </row>
     <row r="941" ht="18.0" customHeight="1">
-      <c r="A941" s="6"/>
+      <c r="A941" s="6" t="s">
+        <v>1511</v>
+      </c>
       <c r="B941" s="17"/>
       <c r="C941" s="14"/>
       <c r="D941" s="22"/>
@@ -45728,7 +46317,9 @@
       <c r="R941" s="7"/>
     </row>
     <row r="942" ht="18.0" customHeight="1">
-      <c r="A942" s="6"/>
+      <c r="A942" s="6" t="s">
+        <v>1512</v>
+      </c>
       <c r="B942" s="17"/>
       <c r="C942" s="14"/>
       <c r="D942" s="22"/>
@@ -45754,7 +46345,9 @@
       <c r="R942" s="7"/>
     </row>
     <row r="943" ht="18.0" customHeight="1">
-      <c r="A943" s="6"/>
+      <c r="A943" s="6" t="s">
+        <v>1513</v>
+      </c>
       <c r="B943" s="17"/>
       <c r="C943" s="14"/>
       <c r="D943" s="22"/>
@@ -45780,7 +46373,9 @@
       <c r="R943" s="7"/>
     </row>
     <row r="944" ht="18.0" customHeight="1">
-      <c r="A944" s="6"/>
+      <c r="A944" s="6" t="s">
+        <v>1514</v>
+      </c>
       <c r="B944" s="17"/>
       <c r="C944" s="14"/>
       <c r="D944" s="22"/>

</xml_diff>